<commit_message>
auto update 2026-10-10 00:09:39
</commit_message>
<xml_diff>
--- a/output/源清单.xlsx
+++ b/output/源清单.xlsx
@@ -4641,17 +4641,17 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>分类实测</t>
+          <t>域名/标记</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>存活</t>
+          <t>失活</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>18禁/动漫</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -4660,13 +4660,9 @@
         </is>
       </c>
       <c r="J72" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="K72" s="2" t="inlineStr">
-        <is>
-          <t>国产情色 | 日本无码 | AV明星 | 中文字幕 | 网红主播 | 成人动漫 | 欧美情色 | 国模私拍 | 长腿丝袜 | 邻家人妻 | 韩国伦理 | 香港伦理 | 精品推荐 | 原纱央莉 | 柚木TINA | 大桥未久 | AV明星1 | 仁科百华 | 天海翼 | 小川阿佐美</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr">
         <is>
           <t>仓库1-增强版,sp696</t>
@@ -6629,17 +6625,17 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>域名/标记</t>
+          <t>上游标记</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>存活/非标准</t>
+          <t>存活</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>动漫/影视/短剧</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr">
@@ -6648,9 +6644,13 @@
         </is>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K107" s="2" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="K107" s="2" t="inlineStr">
+        <is>
+          <t>国产区 | AV区 | 欧美区 | 动漫区 | 网红主播 | 国产传媒 | 探花系列 | 人妻熟女 | 日本无码 | 美乳巨乳 | 强制侵犯 | 制服诱惑 | 绝色佳人 | 风俗泡泡浴 | 家庭乱伦 | AV解说 | 三级电影 | 少女萝莉 | SM调教 | 绝顶潮吹</t>
+        </is>
+      </c>
       <c r="L107" s="2" t="inlineStr">
         <is>
           <t>sp696</t>
@@ -8637,17 +8637,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>分类实测</t>
+          <t>域名/标记</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>存活</t>
+          <t>失活</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>18禁/动漫</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -8656,13 +8656,9 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>7</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>国产情色 | 日本无码 | AV明星 | 中文字幕 | 网红主播 | 成人动漫 | 欧美情色 | 国模私拍 | 长腿丝袜 | 邻家人妻 | 韩国伦理 | 香港伦理 | 精品推荐 | 原纱央莉 | 柚木TINA | 大桥未久 | AV明星1 | 仁科百华 | 天海翼 | 小川阿佐美</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>仓库1-增强版,sp696</t>
@@ -9085,17 +9081,17 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>域名/标记</t>
+          <t>上游标记</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>存活/非标准</t>
+          <t>存活</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>综合</t>
+          <t>动漫/影视/短剧</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -9104,9 +9100,13 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="inlineStr"/>
+        <v>9</v>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>国产区 | AV区 | 欧美区 | 动漫区 | 网红主播 | 国产传媒 | 探花系列 | 人妻熟女 | 日本无码 | 美乳巨乳 | 强制侵犯 | 制服诱惑 | 绝色佳人 | 风俗泡泡浴 | 家庭乱伦 | AV解说 | 三级电影 | 少女萝莉 | SM调教 | 绝顶潮吹</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>sp696</t>

</xml_diff>

<commit_message>
auto update 2026-10-10 00:12:33
</commit_message>
<xml_diff>
--- a/output/源清单.xlsx
+++ b/output/源清单.xlsx
@@ -4641,17 +4641,17 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>域名/标记</t>
+          <t>分类实测</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>失活</t>
+          <t>存活</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18禁/动漫</t>
         </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
@@ -4660,9 +4660,13 @@
         </is>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K72" s="2" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>国产情色 | 日本无码 | AV明星 | 中文字幕 | 网红主播 | 成人动漫 | 欧美情色 | 国模私拍 | 长腿丝袜 | 邻家人妻 | 韩国伦理 | 香港伦理 | 精品推荐 | 原纱央莉 | 柚木TINA | 大桥未久 | AV明星1 | 仁科百华 | 天海翼 | 小川阿佐美</t>
+        </is>
+      </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
           <t>仓库1-增强版,sp696</t>
@@ -8637,17 +8641,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>域名/标记</t>
+          <t>分类实测</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>失活</t>
+          <t>存活</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>18禁/动漫</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -8656,9 +8660,13 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>国产情色 | 日本无码 | AV明星 | 中文字幕 | 网红主播 | 成人动漫 | 欧美情色 | 国模私拍 | 长腿丝袜 | 邻家人妻 | 韩国伦理 | 香港伦理 | 精品推荐 | 原纱央莉 | 柚木TINA | 大桥未久 | AV明星1 | 仁科百华 | 天海翼 | 小川阿佐美</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>仓库1-增强版,sp696</t>

</xml_diff>

<commit_message>
auto update 2026-10-10 00:23:02
</commit_message>
<xml_diff>
--- a/output/源清单.xlsx
+++ b/output/源清单.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1361</v>
+        <v>798</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>265</v>
+        <v>72</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2277</v>
+        <v>2249</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>7679</v>
+        <v>280</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>5053</v>
+        <v>269</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>507</v>
+        <v>425</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>87</v>
+        <v>429</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>677</v>
+        <v>416</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>497</v>
+        <v>232</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>504</v>
+        <v>266</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>4002</v>
+        <v>6811</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>476</v>
+        <v>382</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>270</v>
+        <v>436</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>281</v>
+        <v>57</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1719,7 +1719,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>646</v>
+        <v>415</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>860</v>
+        <v>978</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>830</v>
+        <v>804</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>821</v>
+        <v>719</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>395</v>
+        <v>378</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2024,7 +2024,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>233</v>
+        <v>87</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>364</v>
+        <v>138</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1567</v>
+        <v>1085</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>436</v>
+        <v>385</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>1074</v>
+        <v>324</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2395,7 +2395,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>604</v>
+        <v>419</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>857</v>
+        <v>791</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>302</v>
+        <v>59</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>367</v>
+        <v>213</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>6352</v>
+        <v>1174</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>894</v>
+        <v>209</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>658</v>
+        <v>636</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>452</v>
+        <v>255</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>708</v>
+        <v>597</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>525</v>
+        <v>388</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -3085,7 +3085,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>713</v>
+        <v>538</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -3148,7 +3148,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>439</v>
+        <v>230</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>435</v>
+        <v>365</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -3274,7 +3274,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>3344</v>
+        <v>1863</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>748</v>
+        <v>832</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -3520,7 +3520,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>816</v>
+        <v>824</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>169</v>
+        <v>143</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -3641,7 +3641,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>179</v>
+        <v>144</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H53" s="2" t="n">
-        <v>643</v>
+        <v>1001</v>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
@@ -3819,7 +3819,7 @@
         </is>
       </c>
       <c r="H55" s="2" t="n">
-        <v>379</v>
+        <v>64</v>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
@@ -3882,7 +3882,7 @@
         </is>
       </c>
       <c r="H56" s="2" t="n">
-        <v>780</v>
+        <v>685</v>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
@@ -3945,7 +3945,7 @@
         </is>
       </c>
       <c r="H57" s="2" t="n">
-        <v>842</v>
+        <v>719</v>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
         </is>
       </c>
       <c r="H58" s="2" t="n">
-        <v>803</v>
+        <v>576</v>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="H59" s="2" t="n">
-        <v>1602</v>
+        <v>2148</v>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
@@ -4134,7 +4134,7 @@
         </is>
       </c>
       <c r="H60" s="2" t="n">
-        <v>699</v>
+        <v>355</v>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="H61" s="2" t="n">
-        <v>948</v>
+        <v>586</v>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
@@ -4256,7 +4256,7 @@
         </is>
       </c>
       <c r="H62" s="2" t="n">
-        <v>486</v>
+        <v>385</v>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="H63" s="2" t="n">
-        <v>758</v>
+        <v>610</v>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="H64" s="2" t="n">
-        <v>854</v>
+        <v>1013</v>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
@@ -4441,7 +4441,7 @@
         </is>
       </c>
       <c r="H65" s="2" t="n">
-        <v>581</v>
+        <v>394</v>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
@@ -4504,7 +4504,7 @@
         </is>
       </c>
       <c r="H66" s="2" t="n">
-        <v>4097</v>
+        <v>592</v>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H67" s="2" t="n">
-        <v>626</v>
+        <v>497</v>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
         </is>
       </c>
       <c r="H70" s="2" t="n">
-        <v>753</v>
+        <v>802</v>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="H71" s="2" t="n">
-        <v>773</v>
+        <v>985</v>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
@@ -4861,20 +4861,22 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>分类实测</t>
+          <t>域名/标记</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>存活</t>
-        </is>
-      </c>
-      <c r="H72" s="2" t="n">
-        <v>3585</v>
+          <t>失活</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>18禁/动漫</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
@@ -4883,13 +4885,9 @@
         </is>
       </c>
       <c r="K72" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="L72" s="2" t="inlineStr">
-        <is>
-          <t>国产情色 | 日本无码 | AV明星 | 中文字幕 | 网红主播 | 成人动漫 | 欧美情色 | 国模私拍 | 长腿丝袜 | 邻家人妻 | 韩国伦理 | 香港伦理 | 精品推荐 | 原纱央莉 | 柚木TINA | 大桥未久 | AV明星1 | 仁科百华 | 天海翼 | 小川阿佐美</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L72" s="2" t="inlineStr"/>
       <c r="M72" s="2" t="inlineStr">
         <is>
           <t>仓库1-增强版,sp696</t>
@@ -4933,7 +4931,7 @@
         </is>
       </c>
       <c r="H73" s="2" t="n">
-        <v>1774</v>
+        <v>455</v>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
@@ -4992,7 +4990,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>3547</v>
+        <v>871</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
@@ -5055,7 +5053,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>416</v>
+        <v>174</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -5171,7 +5169,7 @@
         </is>
       </c>
       <c r="H77" s="2" t="n">
-        <v>712</v>
+        <v>556</v>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
@@ -5394,7 +5392,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
@@ -5457,7 +5455,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>415</v>
+        <v>382</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
@@ -5515,7 +5513,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>369</v>
+        <v>350</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -5683,7 +5681,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>510</v>
+        <v>495</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
@@ -5737,7 +5735,7 @@
         </is>
       </c>
       <c r="H87" s="2" t="n">
-        <v>459</v>
+        <v>293</v>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
@@ -5800,7 +5798,7 @@
         </is>
       </c>
       <c r="H88" s="2" t="n">
-        <v>290</v>
+        <v>611</v>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
@@ -5858,7 +5856,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
@@ -5912,7 +5910,7 @@
         </is>
       </c>
       <c r="H90" s="2" t="n">
-        <v>756</v>
+        <v>702</v>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
@@ -5966,7 +5964,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>383</v>
+        <v>723</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
@@ -6024,7 +6022,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>1811</v>
+        <v>2725</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
@@ -6087,7 +6085,7 @@
         </is>
       </c>
       <c r="H93" s="2" t="n">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
@@ -6201,7 +6199,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>1303</v>
+        <v>327</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
@@ -6264,7 +6262,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>379</v>
+        <v>393</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
@@ -6327,7 +6325,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>583</v>
+        <v>556</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
@@ -6390,7 +6388,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>589</v>
+        <v>366</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
@@ -6453,7 +6451,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>756</v>
+        <v>565</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
@@ -6516,7 +6514,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>617</v>
+        <v>661</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
@@ -6579,7 +6577,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>1068</v>
+        <v>749</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
@@ -6642,7 +6640,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>254</v>
+        <v>105</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
@@ -6705,7 +6703,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>2810</v>
+        <v>2345</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
@@ -6768,7 +6766,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>2299</v>
+        <v>2722</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
@@ -6831,7 +6829,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>505</v>
+        <v>310</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
@@ -6894,7 +6892,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>547</v>
+        <v>766</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
@@ -6957,7 +6955,7 @@
         </is>
       </c>
       <c r="H107" s="2" t="n">
-        <v>407</v>
+        <v>273</v>
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
@@ -7020,7 +7018,7 @@
         </is>
       </c>
       <c r="H108" s="2" t="n">
-        <v>707</v>
+        <v>543</v>
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
@@ -7083,7 +7081,7 @@
         </is>
       </c>
       <c r="H109" s="2" t="n">
-        <v>805</v>
+        <v>366</v>
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
@@ -7146,7 +7144,7 @@
         </is>
       </c>
       <c r="H110" s="2" t="n">
-        <v>364</v>
+        <v>340</v>
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
@@ -7209,7 +7207,7 @@
         </is>
       </c>
       <c r="H111" s="2" t="n">
-        <v>542</v>
+        <v>323</v>
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
@@ -7272,7 +7270,7 @@
         </is>
       </c>
       <c r="H112" s="2" t="n">
-        <v>808</v>
+        <v>691</v>
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
@@ -7398,7 +7396,7 @@
         </is>
       </c>
       <c r="H114" s="2" t="n">
-        <v>605</v>
+        <v>447</v>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
@@ -7522,7 +7520,7 @@
         </is>
       </c>
       <c r="H116" s="2" t="n">
-        <v>593</v>
+        <v>486</v>
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
@@ -7585,7 +7583,7 @@
         </is>
       </c>
       <c r="H117" s="2" t="n">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
@@ -7644,7 +7642,7 @@
         </is>
       </c>
       <c r="H118" s="2" t="n">
-        <v>758</v>
+        <v>236</v>
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
@@ -7788,7 +7786,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>265</v>
+        <v>72</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -7911,7 +7909,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>643</v>
+        <v>1001</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -8029,7 +8027,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>379</v>
+        <v>64</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -8092,7 +8090,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>780</v>
+        <v>685</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -8155,7 +8153,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>842</v>
+        <v>719</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -8218,7 +8216,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>803</v>
+        <v>576</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -8281,7 +8279,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1602</v>
+        <v>2148</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -8344,7 +8342,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>699</v>
+        <v>355</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -8407,7 +8405,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>948</v>
+        <v>586</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -8465,7 +8463,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>486</v>
+        <v>385</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -8528,7 +8526,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>758</v>
+        <v>610</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -8591,7 +8589,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>854</v>
+        <v>1013</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -8649,7 +8647,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>581</v>
+        <v>394</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -8712,7 +8710,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>4097</v>
+        <v>592</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -8770,7 +8768,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>626</v>
+        <v>497</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -8953,7 +8951,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>753</v>
+        <v>802</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -9016,7 +9014,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>773</v>
+        <v>985</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -9065,20 +9063,22 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>分类实测</t>
+          <t>域名/标记</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>存活</t>
-        </is>
-      </c>
-      <c r="H23" t="n">
-        <v>3585</v>
+          <t>失活</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>18禁/动漫</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -9087,12 +9087,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>7</v>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>国产情色 | 日本无码 | AV明星 | 中文字幕 | 网红主播 | 成人动漫 | 欧美情色 | 国模私拍 | 长腿丝袜 | 邻家人妻 | 韩国伦理 | 香港伦理 | 精品推荐 | 原纱央莉 | 柚木TINA | 大桥未久 | AV明星1 | 仁科百华 | 天海翼 | 小川阿佐美</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
@@ -9137,7 +9132,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>1774</v>
+        <v>455</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -9245,7 +9240,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>712</v>
+        <v>556</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -9303,7 +9298,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>459</v>
+        <v>293</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -9366,7 +9361,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>290</v>
+        <v>611</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -9424,7 +9419,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>756</v>
+        <v>702</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -9482,7 +9477,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -9540,7 +9535,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>407</v>
+        <v>273</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -9603,7 +9598,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>707</v>
+        <v>543</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -9666,7 +9661,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>805</v>
+        <v>366</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -9729,7 +9724,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>364</v>
+        <v>340</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -9792,7 +9787,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>542</v>
+        <v>323</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -9855,7 +9850,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>808</v>
+        <v>691</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -9981,7 +9976,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>605</v>
+        <v>447</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -10104,7 +10099,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>593</v>
+        <v>486</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -10167,7 +10162,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -10225,7 +10220,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>758</v>
+        <v>236</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -10262,7 +10257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10310,12 +10305,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TV-如意资源</t>
+          <t>如意资源(代理)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://cj.rycjapi.com/api.php/provide/vod</t>
+          <t>https://pz.v88.qzz.io/?url=https://cj.rycjapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -10329,10 +10324,10 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6564</v>
+        <v>1725</v>
       </c>
       <c r="F2" t="n">
-        <v>377</v>
+        <v>390</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -10341,19 +10336,19 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>如意资源(代理)</t>
+          <t>TV-360资源</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://pz.v88.qzz.io/?url=https://cj.rycjapi.com/api.php/provide/vod</t>
+          <t>https://360zy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10363,14 +10358,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>霹雳英雄战纪之塗附世界</t>
+          <t>某暗部的少女共栖</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3648</v>
+        <v>1354</v>
       </c>
       <c r="F3" t="n">
-        <v>341</v>
+        <v>266</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -10379,19 +10374,19 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TV-360资源</t>
+          <t>TV-百度云资源</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://360zy.com/api.php/provide/vod</t>
+          <t>https://api.apibdzy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -10401,23 +10396,23 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>某暗部的少女共栖</t>
+          <t>玄苍路之初入宗门</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1288</v>
+        <v>277</v>
       </c>
       <c r="F4" t="n">
-        <v>277</v>
+        <v>244</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>慢</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -10443,10 +10438,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>505</v>
+        <v>556</v>
       </c>
       <c r="F5" t="n">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -10481,10 +10476,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>511</v>
+        <v>527</v>
       </c>
       <c r="F6" t="n">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -10519,10 +10514,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>541</v>
+        <v>548</v>
       </c>
       <c r="F7" t="n">
-        <v>186</v>
+        <v>203</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -10538,12 +10533,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>iqiyi资源</t>
+          <t>🎬猫眼资源</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.iqiyizyapi.com/api.php/provide/vod</t>
+          <t>https://api.maoyanapi.top/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -10553,14 +10548,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>万物生灵第七季</t>
+          <t>斗罗大陆Ⅱ绝世唐门</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2845</v>
+        <v>716</v>
       </c>
       <c r="F8" t="n">
-        <v>178</v>
+        <v>145</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -10576,12 +10571,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TV-百度云资源</t>
+          <t>TV-樱花资源</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://api.apibdzy.com/api.php/provide/vod</t>
+          <t>https://m3u8.apiyhzy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -10591,14 +10586,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>玄苍路之初入宗门</t>
+          <t>裴太太柔弱人设又翻车了</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>416</v>
+        <v>274</v>
       </c>
       <c r="F9" t="n">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -10633,10 +10628,10 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1641</v>
+        <v>1592</v>
       </c>
       <c r="F10" t="n">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -10652,12 +10647,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TV-樱花资源</t>
+          <t>iqiyi资源</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://m3u8.apiyhzy.com/api.php/provide/vod</t>
+          <t>https://www.iqiyizyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -10667,14 +10662,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>裴太太柔弱人设又翻车了</t>
+          <t>万物生灵第七季</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>133</v>
+        <v>1724</v>
       </c>
       <c r="F11" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -10683,19 +10678,19 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TV-魔都动漫</t>
+          <t>TV-如意资源</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://caiji.moduapi.cc/api.php/provide/vod</t>
+          <t>https://cj.rycjapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -10705,14 +10700,14 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>某暗部的少女共栖</t>
+          <t>霹雳英雄战纪之塗附世界</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>1235</v>
+        <v>3268</v>
       </c>
       <c r="F12" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -10721,19 +10716,19 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TV-魔都资源</t>
+          <t>TV-魔都动漫</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://www.mdzyapi.com/api.php/provide/vod</t>
+          <t>https://caiji.moduapi.cc/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -10747,7 +10742,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>1207</v>
+        <v>719</v>
       </c>
       <c r="F13" t="n">
         <v>62</v>
@@ -10766,12 +10761,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TV-光速资源</t>
+          <t>TV-魔都资源</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://api.guangsuapi.com/api.php/provide/vod</t>
+          <t>https://www.mdzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -10781,22 +10776,18 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>某暗部的少女共栖</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>651</v>
+      </c>
+      <c r="F14" t="n">
+        <v>62</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>慢</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -10850,12 +10841,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TV-U酷资源</t>
+          <t>TV-光速资源</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://api.ukuapi.com/api.php/provide/vod</t>
+          <t>https://api.guangsuapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -10865,7 +10856,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>谋杀奇闻 第一季</t>
+          <t>方舟一号第三季</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -10892,12 +10883,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TV-U酷资源88</t>
+          <t>TV-无尽资源</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://api.ukuapi88.com/api.php/provide/vod</t>
+          <t>https://api.wujinapi.me/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -10907,13 +10898,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>谋杀奇闻 第一季</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>穿越时空甩掉你</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>58</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -10922,7 +10911,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -10934,12 +10923,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TV-步步高资源</t>
+          <t>TV-wujinapi无尽</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://api.yparse.com/api/json</t>
+          <t>https://api.wujinapi.cc/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -10949,13 +10938,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Word is Bond</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>穿越时空甩掉你</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>46</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -10964,7 +10951,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -10995,7 +10982,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>457</v>
+        <v>57</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -11016,12 +11003,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TV-最大资源</t>
+          <t>TV-U酷资源88</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://api.zuidapi.com/api.php/provide/vod</t>
+          <t>https://api.ukuapi88.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -11031,11 +11018,13 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>74</v>
+          <t>谋杀奇闻 第一季</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -11044,7 +11033,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -11056,12 +11045,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TV-无尽资源</t>
+          <t>TV-U酷资源</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://api.wujinapi.me/api.php/provide/vod</t>
+          <t>https://api.ukuapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -11071,11 +11060,13 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>穿越时空甩掉你</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>60</v>
+          <t>谋杀奇闻 第一季</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -11084,7 +11075,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -11096,12 +11087,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TV-wujinapi无尽</t>
+          <t>TV-无尽资源</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://api.wujinapi.cc/api.php/provide/vod</t>
+          <t>https://api.wujinapi.net/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -11115,7 +11106,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>446</v>
+        <v>429</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -11136,12 +11127,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TV-最大点播</t>
+          <t>TV-最大资源</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>http://zuidazy.me/api.php/provide/vod</t>
+          <t>https://api.zuidapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -11155,7 +11146,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>677</v>
+        <v>74</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -11218,12 +11209,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TV-红牛资源</t>
+          <t>TV-丫丫点播</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.hongniuzy2.com/api.php/provide/vod</t>
+          <t>https://cj.yayazy.net/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -11233,13 +11224,11 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>药屋少女的呢喃第三季</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>可以爱你吗</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>684</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -11248,7 +11237,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -11260,12 +11249,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TV-虎牙资源</t>
+          <t>TV-红牛资源</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.huyaapi.com/api.php/provide/vod</t>
+          <t>https://www.hongniuzy2.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -11275,7 +11264,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>南瓜头怪2</t>
+          <t>药屋少女的呢喃第三季</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -11302,12 +11291,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TV-无尽资源</t>
+          <t>TV-牛牛点播</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://api.wujinapi.net/api.php/provide/vod</t>
+          <t>https://api.niuniuzy.me/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -11317,11 +11306,11 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>穿越时空甩掉你</t>
+          <t>可以爱你吗</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>432</v>
+        <v>548</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -11342,12 +11331,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TV-丫丫点播</t>
+          <t>TV-步步高资源</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://cj.yayazy.net/api.php/provide/vod</t>
+          <t>https://api.yparse.com/api/json</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -11357,11 +11346,13 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>766</v>
+          <t>Word is Bond</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -11370,7 +11361,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -11382,12 +11373,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TV-豪华资源</t>
+          <t>TV-索尼资源</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://hhzyapi.com/api.php/provide/vod</t>
+          <t>https://suoniapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -11397,13 +11388,11 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>改造旧冷库后我住成了大别墅</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>70</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -11412,7 +11401,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -11424,12 +11413,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TV-速博资源</t>
+          <t>TV-虎牙资源</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://subocaiji.com/api.php/provide/vod</t>
+          <t>https://www.huyaapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -11439,7 +11428,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
+          <t>南瓜头怪2</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -11466,12 +11455,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TV-金鹰资源</t>
+          <t>TV-速博资源</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://jyzyapi.com/api.php/provide/vod</t>
+          <t>https://subocaiji.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -11508,12 +11497,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TV-量子资源</t>
+          <t>TV-最大点播</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://cj.lziapi.com/api.php/provide/vod</t>
+          <t>http://zuidazy.me/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -11523,13 +11512,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>霹雳英雄战纪之塗附世界</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>可以爱你吗</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>712</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -11538,7 +11525,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -11550,12 +11537,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TV-豆瓣资源</t>
+          <t>TV-暴风资源</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://dbzy.tv/api.php/provide/vod</t>
+          <t>https://bfzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -11565,13 +11552,11 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>骑士情缘</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>乌鸦俱乐部</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1381</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -11580,24 +11565,24 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TV-金鹰点播</t>
+          <t>TV-豆瓣资源</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://jinyingzy.com/api.php/provide/vod</t>
+          <t>https://dbzy.tv/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -11607,7 +11592,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
+          <t>骑士情缘</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -11627,19 +11612,19 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TV-索尼资源</t>
+          <t>TV-量子资源</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://suoniapi.com/api.php/provide/vod</t>
+          <t>https://cj.lziapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -11649,11 +11634,13 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>改造旧冷库后我住成了大别墅</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>52</v>
+          <t>霹雳英雄战纪之塗附世界</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -11662,7 +11649,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -11674,12 +11661,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TV-闪电资源</t>
+          <t>TV-金鹰资源</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://sdzyapi.com/api.php/provide/vod</t>
+          <t>https://jyzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -11689,11 +11676,13 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>728</v>
+          <t>方舟一号第三季</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -11702,7 +11691,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -11714,12 +11703,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TV-牛牛点播</t>
+          <t>TV-金鹰点播</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://api.niuniuzy.me/api.php/provide/vod</t>
+          <t>https://jinyingzy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -11729,11 +11718,13 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>731</v>
+          <t>方舟一号第三季</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -11742,7 +11733,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -11754,12 +11745,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TV-非凡资源</t>
+          <t>TV-豪华资源</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://cj.ffzyapi.com/api.php/provide/vod</t>
+          <t>https://hhzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -11769,7 +11760,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>我家的弟弟们真是让您费心了</t>
+          <t>方舟一号第三季</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -11789,19 +11780,19 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TV-暴风资源</t>
+          <t>TV-非凡资源</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://bfzyapi.com/api.php/provide/vod</t>
+          <t>https://cj.ffzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -11811,11 +11802,13 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>乌鸦俱乐部</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>716</v>
+          <t>我家的弟弟们真是让您费心了</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -11824,24 +11817,24 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TV-1080资源</t>
+          <t>🎬极速资源</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://api.1080zyku.com/inc/api_mac10.php</t>
+          <t>https://jszyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -11851,11 +11844,13 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>冰雪狙击</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>730</v>
+          <t>方舟一号第三季</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -11864,24 +11859,24 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TV-天涯资源</t>
+          <t>红牛资源3</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://tyyszy.com/api.php/provide/vod</t>
+          <t>https://www.hongniuzy3.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -11891,11 +11886,13 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>改造旧冷库后我住成了大别墅</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>264</v>
+          <t>药屋少女的呢喃第三季</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -11904,24 +11901,24 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>失败:ReadTimeout</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>🎬极速资源</t>
+          <t>金鹰资源采集网</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://jszyapi.com/api.php/provide/vod</t>
+          <t>https://jyzyapi.com/provide/vod</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -11958,12 +11955,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>金鹰资源采集网</t>
+          <t>非凡影视new</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://jyzyapi.com/provide/vod</t>
+          <t>https://api.ffzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -11973,7 +11970,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
+          <t>我家的弟弟们真是让您费心了</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -11993,19 +11990,19 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>红牛资源3</t>
+          <t>TV-神马云</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.hongniuzy3.com/api.php/provide/vod</t>
+          <t>https://api.1080zyku.com/inc/apijson.php</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -12015,13 +12012,11 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>药屋少女的呢喃第三季</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>绿头苍蝇</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>707</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -12030,7 +12025,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -12042,12 +12037,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>非凡影视new</t>
+          <t>非凡影视</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://api.ffzyapi.com/api.php/provide/vod</t>
+          <t>http://ffzy5.tv/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -12084,12 +12079,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>非凡影视</t>
+          <t>索尼-闪电资源</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>http://ffzy5.tv/api.php/provide/vod</t>
+          <t>https://xsd.sdzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -12099,13 +12094,11 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>我家的弟弟们真是让您费心了</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>可以爱你吗</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>698</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -12114,24 +12107,24 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>豪华资源(代理)</t>
+          <t>TV-天涯资源</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://pz.v88.qzz.io/?url=https://hhzyapi.com/api.php/provide/vod</t>
+          <t>https://tyyszy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -12141,13 +12134,11 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>改造旧冷库后我住成了大别墅</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>251</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -12156,7 +12147,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>失败:ReadTimeout</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -12210,12 +12201,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>索尼-闪电资源</t>
+          <t>豪华资源(代理)</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://xsd.sdzyapi.com/api.php/provide/vod</t>
+          <t>https://pz.v88.qzz.io/?url=https://hhzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -12225,11 +12216,13 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>702</v>
+          <t>方舟一号第三季</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -12238,7 +12231,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -12334,12 +12327,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TV-神马云</t>
+          <t>🎬快车资源</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://api.1080zyku.com/inc/apijson.php</t>
+          <t>https://caiji.kuaichezy.org/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -12349,11 +12342,11 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>绿头苍蝇</t>
+          <t>可以爱你吗</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>661</v>
+        <v>701</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -12367,19 +12360,19 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>🎬360 资源</t>
+          <t>TV-1080资源</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://360zyzz.com/api.php/provide/vod</t>
+          <t>https://api.1080zyku.com/inc/api_mac10.php</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -12389,11 +12382,11 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Doctor X：白色黑手党时代</t>
+          <t>冰雪狙击</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>621</v>
+        <v>563</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -12402,7 +12395,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>失败:ConnectionError</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -12414,12 +12407,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>🎬快车资源</t>
+          <t>🎬360 资源</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://caiji.kuaichezy.org/api.php/provide/vod</t>
+          <t>https://360zyzz.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -12429,11 +12422,11 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
+          <t>Doctor X：白色黑手党时代</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>733</v>
+        <v>613</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -12447,19 +12440,19 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>艾旦影视(代理)</t>
+          <t>TV-闪电资源</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://pz.v88.qzz.io/?url=https://lovedan.net/api.php/provide/vod</t>
+          <t>https://sdzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -12469,11 +12462,11 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>伟大的长征</t>
+          <t>可以爱你吗</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>3497</v>
+        <v>725</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -12482,7 +12475,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>失败:ReadTimeout</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -12534,12 +12527,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>🎬猫眼资源</t>
+          <t>艾旦影视(代理)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://api.maoyanapi.top/api.php/provide/vod</t>
+          <t>https://pz.v88.qzz.io/?url=https://lovedan.net/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -12547,11 +12540,13 @@
           <t>否</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>伟大的长征</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1647</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -12560,24 +12555,24 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>失败:ReadTimeout</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>AV-森林资源</t>
+          <t>🔞森林资源</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://slapibf.com/api.php/provide/vod</t>
+          <t>https://beiyong.slapibf.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -12591,10 +12586,10 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>492</v>
+        <v>538</v>
       </c>
       <c r="F58" t="n">
-        <v>11175</v>
+        <v>11489</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -12610,12 +12605,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>🔞森林资源</t>
+          <t>AV-155资源</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://beiyong.slapibf.com/api.php/provide/vod</t>
+          <t>https://155api.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -12625,14 +12620,14 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>FTHTD-144FALENO学校训练营公共浴池</t>
+          <t>内裤走光后宫学园只有我一MOODYZ大崎広浩治沙</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>559</v>
+        <v>53</v>
       </c>
       <c r="F59" t="n">
-        <v>10991</v>
+        <v>11223</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -12648,12 +12643,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AV-155资源</t>
+          <t>AV-森林资源</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://155api.com/api.php/provide/vod</t>
+          <t>https://slapibf.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -12663,14 +12658,14 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>内裤走光后宫学园只有我一MOODYZ大崎広浩治沙</t>
+          <t>FTHTD-144FALENO学校训练营公共浴池</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>55</v>
+        <v>491</v>
       </c>
       <c r="F60" t="n">
-        <v>9523</v>
+        <v>11051</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -12686,12 +12681,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>🔞杏吧资源</t>
+          <t>AV-辣椒资源</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://xingba222.com/api.php/provide/vod</t>
+          <t>https://apilj.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -12701,14 +12696,14 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">DASS-303 被派遣按摩師 按摩到敏感部位 </t>
+          <t>泌尿科的美人女医8人プラネットプラス伊织凉子,管</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>476</v>
+        <v>4034</v>
       </c>
       <c r="F61" t="n">
-        <v>7670</v>
+        <v>9088</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -12717,19 +12712,19 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>性吧资源</t>
+          <t>🔞杏吧资源</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>https://xingba111.com/api.php/provide/vod</t>
+          <t>https://xingba222.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -12743,10 +12738,10 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>621</v>
+        <v>456</v>
       </c>
       <c r="F62" t="n">
-        <v>7620</v>
+        <v>7835</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -12781,10 +12776,10 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>624</v>
+        <v>617</v>
       </c>
       <c r="F63" t="n">
-        <v>6948</v>
+        <v>7485</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -12800,12 +12795,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>AV-鲨鱼资源</t>
+          <t>性吧资源</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://shayuapi.com/api.php/provide/vod</t>
+          <t>https://xingba111.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -12815,14 +12810,14 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>[瘦猴勾搭] 良家人妻被撩到腿软，眼睛妹妹骚穴求</t>
+          <t xml:space="preserve">DASS-303 被派遣按摩師 按摩到敏感部位 </t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>9382</v>
+        <v>552</v>
       </c>
       <c r="F64" t="n">
-        <v>5048</v>
+        <v>6140</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -12831,19 +12826,19 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AV-辣椒资源</t>
+          <t>AV-乐播资源</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://apilj.com/api.php/provide/vod</t>
+          <t>https://lbapi9.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -12853,14 +12848,14 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>泌尿科的美人女医8人プラネットプラス伊织凉子,管</t>
+          <t>[无码] 苗条人妻床上骚劲爆棚，风骚妩媚狂求内射</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>731</v>
+        <v>873</v>
       </c>
       <c r="F65" t="n">
-        <v>4988</v>
+        <v>3360</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -12869,19 +12864,19 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AV-乐播资源</t>
+          <t>🔞滴滴资源</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://lbapi9.com/api.php/provide/vod</t>
+          <t>https://api.ddapi.cc/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -12891,18 +12886,18 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>[无码] 苗条人妻床上骚劲爆棚，风骚妩媚狂求内射</t>
+          <t>双飞学生妹【蔡萝莉】SM捆绑~白丝足交~强制高潮</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>860</v>
+        <v>375</v>
       </c>
       <c r="F66" t="n">
-        <v>2018</v>
+        <v>838</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>快</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -12933,10 +12928,10 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="F67" t="n">
-        <v>895</v>
+        <v>805</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -12952,12 +12947,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>🔞滴滴资源</t>
+          <t>AV-JKUN资源</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://api.ddapi.cc/api.php/provide/vod</t>
+          <t>https://jkunzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -12967,14 +12962,14 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>双飞学生妹【蔡萝莉】SM捆绑~白丝足交~强制高潮</t>
+          <t>pacopacomama-072023_880-</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>376</v>
+        <v>58</v>
       </c>
       <c r="F68" t="n">
-        <v>842</v>
+        <v>640</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -12990,12 +12985,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>AV-JKUN资源</t>
+          <t>AV-玉兔资源</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>https://jkunzyapi.com/api.php/provide/vod</t>
+          <t>https://apiyutu.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -13005,14 +13000,14 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>pacopacomama-072023_880-</t>
+          <t>家庭旅馆偷拍性饥渴嫂子偷情小叔子裤子都没脱就主动</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>69</v>
+        <v>380</v>
       </c>
       <c r="F69" t="n">
-        <v>651</v>
+        <v>463</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -13047,7 +13042,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>583</v>
+        <v>231</v>
       </c>
       <c r="F70" t="n">
         <v>453</v>
@@ -13066,12 +13061,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>AV-玉兔资源</t>
+          <t>AV-精品资源</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://apiyutu.com/api.php/provide/vod</t>
+          <t>https://www.jingpinx.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -13081,14 +13076,14 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>家庭旅馆偷拍性饥渴嫂子偷情小叔子裤子都没脱就主动</t>
+          <t>純潔的輪舞曲_2</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>372</v>
+        <v>397</v>
       </c>
       <c r="F71" t="n">
-        <v>436</v>
+        <v>413</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -13097,19 +13092,19 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>🔞桃花资源</t>
+          <t>AV-奶香香</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://thzy1.me/api.php/provide/vod</t>
+          <t>https://Naixxzy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -13119,14 +13114,14 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>[HornyVerse]_Jane_Doe_Fu</t>
+          <t>[换脸]孙彩瑛 热热的骚逼..</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>475</v>
+        <v>558</v>
       </c>
       <c r="F72" t="n">
-        <v>365</v>
+        <v>295</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -13142,12 +13137,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>AV-奶香香</t>
+          <t>🔞桃花资源</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://Naixxzy.com/api.php/provide/vod</t>
+          <t>https://thzy1.me/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -13157,14 +13152,14 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>[换脸]孙彩瑛 热热的骚逼..</t>
+          <t>[HornyVerse]_Jane_Doe_Fu</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>557</v>
+        <v>611</v>
       </c>
       <c r="F73" t="n">
-        <v>299</v>
+        <v>254</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -13180,12 +13175,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>🔞小鸡资源</t>
+          <t>🔞-大奶子-</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://api.xiaojizy.live/provide/vod</t>
+          <t>https://apidanaizi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -13195,14 +13190,14 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>李素英合3</t>
+          <t>【最新自录-清纯甜美二次元美少女】白裙情趣装罕见</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>357</v>
+        <v>563</v>
       </c>
       <c r="F74" t="n">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -13211,19 +13206,19 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>🔞-大奶子-</t>
+          <t>AV-奥斯卡资源</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://apidanaizi.com/api.php/provide/vod</t>
+          <t>https://aosikazy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -13233,14 +13228,14 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>【最新自录-清纯甜美二次元美少女】白裙情趣装罕见</t>
+          <t>真实与后妈乱伦9个月</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>540</v>
+        <v>624</v>
       </c>
       <c r="F75" t="n">
-        <v>227</v>
+        <v>179</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -13249,19 +13244,19 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>AV-精品资源</t>
+          <t>🔞小鸡资源</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://www.jingpinx.com/api.php/provide/vod</t>
+          <t>https://api.xiaojizy.live/provide/vod</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -13271,14 +13266,14 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>純潔的輪舞曲_2</t>
+          <t>李素英合3</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>392</v>
+        <v>310</v>
       </c>
       <c r="F76" t="n">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -13294,12 +13289,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>AV-奥斯卡资源</t>
+          <t>AV-91麻豆</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>https://aosikazy.com/api.php/provide/vod</t>
+          <t>https://91md.me/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -13309,14 +13304,14 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>真实与后妈乱伦9个月</t>
+          <t>被老师欺负的黑丝女高-桥本香菜</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>655</v>
+        <v>1196</v>
       </c>
       <c r="F77" t="n">
-        <v>184</v>
+        <v>150</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -13325,7 +13320,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -13351,10 +13346,10 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>934</v>
+        <v>981</v>
       </c>
       <c r="F78" t="n">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -13370,12 +13365,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>AV-91麻豆</t>
+          <t>AV-souav资源</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://91md.me/api.php/provide/vod</t>
+          <t>https://api.souavzy.vip/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -13385,18 +13380,20 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>被老师欺负的黑丝女高-桥本香菜</t>
+          <t>白嫩美女月月无套内射初体验</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>1092</v>
-      </c>
-      <c r="F79" t="n">
-        <v>115</v>
+        <v>275</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>慢</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -13408,12 +13405,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>AV-souav资源</t>
+          <t>黄色资源啊啊</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://api.souavzy.vip/api.php/provide/vod</t>
+          <t>https://hsckzy888.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -13423,11 +13420,13 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>白嫩美女月月无套内射初体验</t>
-        </is>
-      </c>
-      <c r="E80" t="n">
-        <v>926</v>
+          <t>公共厕所肉便器 我二话 高岭千佳</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -13436,7 +13435,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -13448,12 +13447,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>黄色资源啊啊</t>
+          <t>🔞黄色仓库</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://hsckzy888.com/api.php/provide/vod</t>
+          <t>https://hsckzy.xyz/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -13490,12 +13489,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>🔞黄色仓库</t>
+          <t>🔞souavZY</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>https://hsckzy.xyz/api.php/provide/vod</t>
+          <t>https://api.souavzyw.net/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -13505,13 +13504,11 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>公共厕所肉便器 我二话 高岭千佳</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>与儿子所在托儿所的巨乳人妻老师缠绵做爱～老师太过</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>456</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -13520,7 +13517,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -13532,12 +13529,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>🔞souavZY</t>
+          <t>🔞色猫资源</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>https://api.souavzyw.net/api.php/provide/vod</t>
+          <t>https://caiji.semaozy.net/inc/apijson_vod.php/provide/vod</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -13545,13 +13542,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>与儿子所在托儿所的巨乳人妻老师缠绵做爱～老师太过</t>
-        </is>
-      </c>
-      <c r="E83" t="n">
-        <v>566</v>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -13560,48 +13555,10 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>🔞色猫资源</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>https://caiji.semaozy.net/inc/apijson_vod.php/provide/vod</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr"/>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>未测出</t>
-        </is>
-      </c>
-      <c r="H84" t="inlineStr">
         <is>
           <t>是</t>
         </is>

</xml_diff>

<commit_message>
auto update 2026-10-10 00:35:05
</commit_message>
<xml_diff>
--- a/output/源清单.xlsx
+++ b/output/源清单.xlsx
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>798</v>
+        <v>1630</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>72</v>
+        <v>251</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -679,7 +679,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2249</v>
+        <v>2071</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>490</v>
+        <v>807</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>280</v>
+        <v>981</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -868,7 +868,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>269</v>
+        <v>454</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>425</v>
+        <v>490</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>429</v>
+        <v>512</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>416</v>
+        <v>611</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>232</v>
+        <v>336</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>266</v>
+        <v>513</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>6811</v>
+        <v>7374</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1535,7 +1535,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>382</v>
+        <v>645</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>436</v>
+        <v>649</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1661,7 +1661,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>57</v>
+        <v>240</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1719,7 +1719,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>415</v>
+        <v>636</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>978</v>
+        <v>841</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>804</v>
+        <v>865</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>719</v>
+        <v>611</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>378</v>
+        <v>423</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -2024,7 +2024,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>87</v>
+        <v>260</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>138</v>
+        <v>335</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2145,7 +2145,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>1085</v>
+        <v>1575</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2208,7 +2208,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>385</v>
+        <v>432</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>324</v>
+        <v>1567</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2395,7 +2395,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>419</v>
+        <v>701</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -2458,7 +2458,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>791</v>
+        <v>1284</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>59</v>
+        <v>196</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>213</v>
+        <v>471</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>1174</v>
+        <v>1154</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -2710,7 +2710,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>209</v>
+        <v>481</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -2833,7 +2833,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>636</v>
+        <v>1017</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -2896,7 +2896,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>255</v>
+        <v>518</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2959,7 +2959,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>597</v>
+        <v>618</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>388</v>
+        <v>586</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -3085,7 +3085,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>538</v>
+        <v>696</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -3148,7 +3148,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>230</v>
+        <v>550</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -3211,7 +3211,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>365</v>
+        <v>511</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -3274,7 +3274,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>1863</v>
+        <v>7141</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>832</v>
+        <v>1027</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -3520,7 +3520,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>824</v>
+        <v>987</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -3583,7 +3583,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>143</v>
+        <v>90</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -3641,7 +3641,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>144</v>
+        <v>105</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H53" s="2" t="n">
-        <v>1001</v>
+        <v>700</v>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
@@ -3819,7 +3819,7 @@
         </is>
       </c>
       <c r="H55" s="2" t="n">
-        <v>64</v>
+        <v>548</v>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
@@ -3882,7 +3882,7 @@
         </is>
       </c>
       <c r="H56" s="2" t="n">
-        <v>685</v>
+        <v>777</v>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
@@ -3945,7 +3945,7 @@
         </is>
       </c>
       <c r="H57" s="2" t="n">
-        <v>719</v>
+        <v>993</v>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
@@ -4008,7 +4008,7 @@
         </is>
       </c>
       <c r="H58" s="2" t="n">
-        <v>576</v>
+        <v>888</v>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
@@ -4071,7 +4071,7 @@
         </is>
       </c>
       <c r="H59" s="2" t="n">
-        <v>2148</v>
+        <v>2925</v>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
@@ -4134,7 +4134,7 @@
         </is>
       </c>
       <c r="H60" s="2" t="n">
-        <v>355</v>
+        <v>784</v>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
@@ -4197,7 +4197,7 @@
         </is>
       </c>
       <c r="H61" s="2" t="n">
-        <v>586</v>
+        <v>854</v>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
@@ -4256,7 +4256,7 @@
         </is>
       </c>
       <c r="H62" s="2" t="n">
-        <v>385</v>
+        <v>577</v>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="H63" s="2" t="n">
-        <v>610</v>
+        <v>743</v>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="H64" s="2" t="n">
-        <v>1013</v>
+        <v>1217</v>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
@@ -4441,7 +4441,7 @@
         </is>
       </c>
       <c r="H65" s="2" t="n">
-        <v>394</v>
+        <v>802</v>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
@@ -4504,7 +4504,7 @@
         </is>
       </c>
       <c r="H66" s="2" t="n">
-        <v>592</v>
+        <v>1323</v>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H67" s="2" t="n">
-        <v>497</v>
+        <v>712</v>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
@@ -4748,7 +4748,7 @@
         </is>
       </c>
       <c r="H70" s="2" t="n">
-        <v>802</v>
+        <v>1509</v>
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
@@ -4811,7 +4811,7 @@
         </is>
       </c>
       <c r="H71" s="2" t="n">
-        <v>985</v>
+        <v>1008</v>
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
@@ -4931,7 +4931,7 @@
         </is>
       </c>
       <c r="H73" s="2" t="n">
-        <v>455</v>
+        <v>663</v>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>871</v>
+        <v>2523</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
@@ -5053,7 +5053,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>174</v>
+        <v>385</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
         </is>
       </c>
       <c r="H77" s="2" t="n">
-        <v>556</v>
+        <v>773</v>
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
@@ -5392,7 +5392,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>573</v>
+        <v>766</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
@@ -5455,7 +5455,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>382</v>
+        <v>588</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
@@ -5513,7 +5513,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>350</v>
+        <v>236</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -5681,7 +5681,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>495</v>
+        <v>521</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
@@ -5735,7 +5735,7 @@
         </is>
       </c>
       <c r="H87" s="2" t="n">
-        <v>293</v>
+        <v>436</v>
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
@@ -5798,7 +5798,7 @@
         </is>
       </c>
       <c r="H88" s="2" t="n">
-        <v>611</v>
+        <v>312</v>
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="I89" t="inlineStr">
         <is>
@@ -5910,7 +5910,7 @@
         </is>
       </c>
       <c r="H90" s="2" t="n">
-        <v>702</v>
+        <v>807</v>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
@@ -5964,7 +5964,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>723</v>
+        <v>575</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
@@ -6013,34 +6013,31 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>分类实测</t>
+          <t>无法探测→按普通处理</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>存活</t>
-        </is>
-      </c>
-      <c r="H92" t="n">
-        <v>2725</v>
+          <t>失活</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>动漫/影视/短剧</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>是(少量)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K92" t="n">
-        <v>1</v>
-      </c>
-      <c r="L92" t="inlineStr">
-        <is>
-          <t>国产动漫 | 日韩动漫 | 欧美动漫 | 港台动漫 | 动漫电影 | 里番动漫 | 电影 | 连续剧 | 综艺 | 动作片 | 喜剧片 | 爱情片 | 科幻片 | 恐怖片 | 剧情片 | 战争片 | 惊悚片 | 家庭片 | 古装片 | 历史片</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -6085,7 +6082,7 @@
         </is>
       </c>
       <c r="H93" s="2" t="n">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
@@ -6199,7 +6196,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>327</v>
+        <v>696</v>
       </c>
       <c r="I95" t="inlineStr">
         <is>
@@ -6262,7 +6259,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>393</v>
+        <v>386</v>
       </c>
       <c r="I96" t="inlineStr">
         <is>
@@ -6325,7 +6322,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>556</v>
+        <v>620</v>
       </c>
       <c r="I97" t="inlineStr">
         <is>
@@ -6388,7 +6385,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>366</v>
+        <v>592</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
@@ -6451,7 +6448,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>565</v>
+        <v>664</v>
       </c>
       <c r="I99" t="inlineStr">
         <is>
@@ -6514,7 +6511,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>661</v>
+        <v>933</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
@@ -6577,7 +6574,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>749</v>
+        <v>737</v>
       </c>
       <c r="I101" t="inlineStr">
         <is>
@@ -6640,7 +6637,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>105</v>
+        <v>252</v>
       </c>
       <c r="I102" t="inlineStr">
         <is>
@@ -6703,7 +6700,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>2345</v>
+        <v>3411</v>
       </c>
       <c r="I103" t="inlineStr">
         <is>
@@ -6766,7 +6763,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>2722</v>
+        <v>1230</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
@@ -6829,7 +6826,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>310</v>
+        <v>420</v>
       </c>
       <c r="I105" t="inlineStr">
         <is>
@@ -6892,7 +6889,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>766</v>
+        <v>825</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
@@ -6955,7 +6952,7 @@
         </is>
       </c>
       <c r="H107" s="2" t="n">
-        <v>273</v>
+        <v>393</v>
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
@@ -7018,7 +7015,7 @@
         </is>
       </c>
       <c r="H108" s="2" t="n">
-        <v>543</v>
+        <v>801</v>
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
@@ -7081,7 +7078,7 @@
         </is>
       </c>
       <c r="H109" s="2" t="n">
-        <v>366</v>
+        <v>707</v>
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
@@ -7144,7 +7141,7 @@
         </is>
       </c>
       <c r="H110" s="2" t="n">
-        <v>340</v>
+        <v>371</v>
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
@@ -7207,7 +7204,7 @@
         </is>
       </c>
       <c r="H111" s="2" t="n">
-        <v>323</v>
+        <v>546</v>
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
@@ -7270,7 +7267,7 @@
         </is>
       </c>
       <c r="H112" s="2" t="n">
-        <v>691</v>
+        <v>1143</v>
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
@@ -7333,7 +7330,7 @@
         </is>
       </c>
       <c r="H113" s="2" t="n">
-        <v>496</v>
+        <v>524</v>
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
@@ -7396,7 +7393,7 @@
         </is>
       </c>
       <c r="H114" s="2" t="n">
-        <v>447</v>
+        <v>2222</v>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
@@ -7520,7 +7517,7 @@
         </is>
       </c>
       <c r="H116" s="2" t="n">
-        <v>486</v>
+        <v>591</v>
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
@@ -7583,7 +7580,7 @@
         </is>
       </c>
       <c r="H117" s="2" t="n">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
@@ -7642,7 +7639,7 @@
         </is>
       </c>
       <c r="H118" s="2" t="n">
-        <v>236</v>
+        <v>709</v>
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
@@ -7786,7 +7783,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>72</v>
+        <v>251</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -7909,7 +7906,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>1001</v>
+        <v>700</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -8027,7 +8024,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>64</v>
+        <v>548</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -8090,7 +8087,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>685</v>
+        <v>777</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -8153,7 +8150,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>719</v>
+        <v>993</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -8216,7 +8213,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>576</v>
+        <v>888</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -8279,7 +8276,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2148</v>
+        <v>2925</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -8342,7 +8339,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>355</v>
+        <v>784</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -8405,7 +8402,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>586</v>
+        <v>854</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -8463,7 +8460,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>385</v>
+        <v>577</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -8526,7 +8523,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>610</v>
+        <v>743</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -8589,7 +8586,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1013</v>
+        <v>1217</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -8647,7 +8644,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>394</v>
+        <v>802</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -8710,7 +8707,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>592</v>
+        <v>1323</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -8768,7 +8765,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>497</v>
+        <v>712</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -8951,7 +8948,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>802</v>
+        <v>1509</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -9014,7 +9011,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>985</v>
+        <v>1008</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -9132,7 +9129,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>455</v>
+        <v>663</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -9240,7 +9237,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>556</v>
+        <v>773</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -9298,7 +9295,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>293</v>
+        <v>436</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -9361,7 +9358,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>611</v>
+        <v>312</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -9419,7 +9416,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>702</v>
+        <v>807</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -9477,7 +9474,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>514</v>
+        <v>522</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -9535,7 +9532,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>273</v>
+        <v>393</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -9598,7 +9595,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>543</v>
+        <v>801</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -9661,7 +9658,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>366</v>
+        <v>707</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -9724,7 +9721,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>340</v>
+        <v>371</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -9787,7 +9784,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>323</v>
+        <v>546</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -9850,7 +9847,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>691</v>
+        <v>1143</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -9913,7 +9910,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>496</v>
+        <v>524</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -9976,7 +9973,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>447</v>
+        <v>2222</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -10099,7 +10096,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>486</v>
+        <v>591</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -10162,7 +10159,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -10220,7 +10217,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>236</v>
+        <v>709</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -10257,7 +10254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H83"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10305,12 +10302,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>如意资源(代理)</t>
+          <t>🎬猫眼资源</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://pz.v88.qzz.io/?url=https://cj.rycjapi.com/api.php/provide/vod</t>
+          <t>https://api.maoyanapi.top/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -10320,14 +10317,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>霹雳英雄战纪之塗附世界</t>
+          <t>斗罗大陆Ⅱ绝世唐门</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1725</v>
+        <v>732</v>
       </c>
       <c r="F2" t="n">
-        <v>390</v>
+        <v>369</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -10336,19 +10333,19 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TV-360资源</t>
+          <t>如意资源(代理)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://360zy.com/api.php/provide/vod</t>
+          <t>https://pz.v88.qzz.io/?url=https://cj.rycjapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -10358,14 +10355,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>某暗部的少女共栖</t>
+          <t>霹雳英雄战纪之塗附世界</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1354</v>
+        <v>1534</v>
       </c>
       <c r="F3" t="n">
-        <v>266</v>
+        <v>324</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -10374,19 +10371,19 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TV-百度云资源</t>
+          <t>TV-360资源</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://api.apibdzy.com/api.php/provide/vod</t>
+          <t>https://360zy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -10396,23 +10393,23 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>玄苍路之初入宗门</t>
+          <t>某暗部的少女共栖</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>277</v>
+        <v>1371</v>
       </c>
       <c r="F4" t="n">
-        <v>244</v>
+        <v>267</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>慢</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
@@ -10438,10 +10435,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>556</v>
+        <v>600</v>
       </c>
       <c r="F5" t="n">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -10476,10 +10473,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>527</v>
+        <v>516</v>
       </c>
       <c r="F6" t="n">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -10495,12 +10492,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TV-ikun资源</t>
+          <t>TV-百度云资源</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://ikunzyapi.com/api.php/provide/vod</t>
+          <t>https://api.apibdzy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -10510,14 +10507,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>某暗部的少女共栖</t>
+          <t>玄苍路之初入宗门</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>548</v>
+        <v>1914</v>
       </c>
       <c r="F7" t="n">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -10533,12 +10530,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>🎬猫眼资源</t>
+          <t>TV-ikun资源</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://api.maoyanapi.top/api.php/provide/vod</t>
+          <t>https://ikunzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -10548,14 +10545,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>斗罗大陆Ⅱ绝世唐门</t>
+          <t>某暗部的少女共栖</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>716</v>
+        <v>519</v>
       </c>
       <c r="F8" t="n">
-        <v>145</v>
+        <v>195</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -10564,19 +10561,19 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TV-樱花资源</t>
+          <t>TV-茅台资源</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://m3u8.apiyhzy.com/api.php/provide/vod</t>
+          <t>https://caiji.maotaizy.cc/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -10586,14 +10583,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>裴太太柔弱人设又翻车了</t>
+          <t>梦想改造家 第13季</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>274</v>
+        <v>1540</v>
       </c>
       <c r="F9" t="n">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -10602,19 +10599,19 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TV-茅台资源</t>
+          <t>TV-如意资源</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://caiji.maotaizy.cc/api.php/provide/vod</t>
+          <t>https://cj.rycjapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -10624,14 +10621,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>梦想改造家 第13季</t>
+          <t>霹雳英雄战纪之塗附世界</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1592</v>
+        <v>4567</v>
       </c>
       <c r="F10" t="n">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -10647,12 +10644,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>iqiyi资源</t>
+          <t>TV-樱花资源</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.iqiyizyapi.com/api.php/provide/vod</t>
+          <t>https://m3u8.apiyhzy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -10662,14 +10659,14 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>万物生灵第七季</t>
+          <t>裴太太柔弱人设又翻车了</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>1724</v>
+        <v>113</v>
       </c>
       <c r="F11" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -10678,19 +10675,19 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TV-如意资源</t>
+          <t>TV-魔都资源</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://cj.rycjapi.com/api.php/provide/vod</t>
+          <t>https://www.mdzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -10700,14 +10697,14 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>霹雳英雄战纪之塗附世界</t>
+          <t>某暗部的少女共栖</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3268</v>
+        <v>974</v>
       </c>
       <c r="F12" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -10716,7 +10713,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -10742,10 +10739,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>719</v>
+        <v>988</v>
       </c>
       <c r="F13" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -10761,12 +10758,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TV-魔都资源</t>
+          <t>TV-U酷资源</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://www.mdzyapi.com/api.php/provide/vod</t>
+          <t>https://api.ukuapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -10776,18 +10773,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>某暗部的少女共栖</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>651</v>
-      </c>
-      <c r="F14" t="n">
-        <v>62</v>
+          <t>谋杀奇闻 第一季</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>慢</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -10799,12 +10800,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TV-新浪点播</t>
+          <t>TV-光速资源</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://api.xinlangapi.com/xinlangapi.php/provide/vod</t>
+          <t>https://api.guangsuapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -10841,12 +10842,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TV-光速资源</t>
+          <t>TV-新浪点播</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://api.guangsuapi.com/api.php/provide/vod</t>
+          <t>https://api.xinlangapi.com/xinlangapi.php/provide/vod</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -10883,12 +10884,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TV-无尽资源</t>
+          <t>TV-U酷资源88</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://api.wujinapi.me/api.php/provide/vod</t>
+          <t>https://api.ukuapi88.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -10898,11 +10899,13 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>穿越时空甩掉你</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>58</v>
+          <t>谋杀奇闻 第一季</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -10911,7 +10914,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -10923,12 +10926,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TV-wujinapi无尽</t>
+          <t>TV-步步高资源</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://api.wujinapi.cc/api.php/provide/vod</t>
+          <t>https://api.yparse.com/api/json</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -10938,11 +10941,13 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>穿越时空甩掉你</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>46</v>
+          <t>Word is Bond</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -10951,7 +10956,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -10963,12 +10968,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TV-无尽资源</t>
+          <t>TV-暴风资源</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://api.wujinapi.com/api.php/provide/vod</t>
+          <t>https://bfzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -10978,11 +10983,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>穿越时空甩掉你</t>
+          <t>乌鸦俱乐部</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>57</v>
+        <v>1025</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -11003,12 +11008,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TV-U酷资源88</t>
+          <t>TV-最大点播</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://api.ukuapi88.com/api.php/provide/vod</t>
+          <t>http://zuidazy.me/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -11018,13 +11023,11 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>谋杀奇闻 第一季</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>可以爱你吗</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>700</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -11033,7 +11036,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -11045,12 +11048,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TV-U酷资源</t>
+          <t>TV-无尽资源</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://api.ukuapi.com/api.php/provide/vod</t>
+          <t>https://api.wujinapi.me/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -11060,13 +11063,11 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>谋杀奇闻 第一季</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>穿越时空甩掉你</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>222</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -11075,7 +11076,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -11092,7 +11093,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://api.wujinapi.net/api.php/provide/vod</t>
+          <t>https://api.wujinapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -11106,7 +11107,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>429</v>
+        <v>417</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -11127,12 +11128,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TV-最大资源</t>
+          <t>TV-无尽资源</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://api.zuidapi.com/api.php/provide/vod</t>
+          <t>https://api.wujinapi.net/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -11142,11 +11143,11 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
+          <t>穿越时空甩掉你</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>74</v>
+        <v>440</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -11167,12 +11168,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TV-电影天堂资源</t>
+          <t>TV-最大资源</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>http://caiji.dyttzyapi.com/api.php/provide/vod</t>
+          <t>https://api.zuidapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -11182,13 +11183,11 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>霹雳英雄战纪之塗附世界</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>可以爱你吗</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>59</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -11197,24 +11196,24 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TV-丫丫点播</t>
+          <t>TV-电影天堂资源</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://cj.yayazy.net/api.php/provide/vod</t>
+          <t>http://caiji.dyttzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -11224,11 +11223,13 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>684</v>
+          <t>霹雳英雄战纪之塗附世界</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -11237,12 +11238,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
@@ -11291,12 +11292,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TV-牛牛点播</t>
+          <t>TV-丫丫点播</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://api.niuniuzy.me/api.php/provide/vod</t>
+          <t>https://cj.yayazy.net/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -11310,7 +11311,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>548</v>
+        <v>751</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -11331,12 +11332,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TV-步步高资源</t>
+          <t>TV-虎牙资源</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://api.yparse.com/api/json</t>
+          <t>https://www.huyaapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -11346,7 +11347,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Word is Bond</t>
+          <t>南瓜头怪2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -11373,12 +11374,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TV-索尼资源</t>
+          <t>TV-豪华资源</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://suoniapi.com/api.php/provide/vod</t>
+          <t>https://hhzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -11388,11 +11389,13 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>改造旧冷库后我住成了大别墅</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>70</v>
+          <t>方舟一号第三季</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -11401,7 +11404,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -11413,12 +11416,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TV-虎牙资源</t>
+          <t>TV-金鹰资源</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.huyaapi.com/api.php/provide/vod</t>
+          <t>https://jyzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -11428,7 +11431,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>南瓜头怪2</t>
+          <t>方舟一号第三季</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -11497,12 +11500,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TV-最大点播</t>
+          <t>TV-wujinapi无尽</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>http://zuidazy.me/api.php/provide/vod</t>
+          <t>https://api.wujinapi.cc/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -11512,11 +11515,11 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
+          <t>穿越时空甩掉你</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>712</v>
+        <v>1273</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -11537,12 +11540,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TV-暴风资源</t>
+          <t>TV-豆瓣资源</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://bfzyapi.com/api.php/provide/vod</t>
+          <t>https://dbzy.tv/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -11552,11 +11555,13 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>乌鸦俱乐部</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>1381</v>
+          <t>骑士情缘</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -11565,24 +11570,24 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TV-豆瓣资源</t>
+          <t>TV-金鹰点播</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://dbzy.tv/api.php/provide/vod</t>
+          <t>https://jinyingzy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -11592,7 +11597,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>骑士情缘</t>
+          <t>方舟一号第三季</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -11612,7 +11617,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -11661,12 +11666,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TV-金鹰资源</t>
+          <t>TV-牛牛点播</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://jyzyapi.com/api.php/provide/vod</t>
+          <t>https://api.niuniuzy.me/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -11676,13 +11681,11 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>可以爱你吗</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>724</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -11691,7 +11694,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -11703,12 +11706,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TV-金鹰点播</t>
+          <t>TV-非凡资源</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://jinyingzy.com/api.php/provide/vod</t>
+          <t>https://cj.ffzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -11718,7 +11721,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
+          <t>金缮</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -11738,19 +11741,19 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TV-豪华资源</t>
+          <t>TV-闪电资源</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://hhzyapi.com/api.php/provide/vod</t>
+          <t>https://sdzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -11760,13 +11763,11 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>可以爱你吗</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>513</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -11775,7 +11776,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -11787,12 +11788,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TV-非凡资源</t>
+          <t>TV-索尼资源</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://cj.ffzyapi.com/api.php/provide/vod</t>
+          <t>https://suoniapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -11802,13 +11803,11 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>我家的弟弟们真是让您费心了</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>改造旧冷库后我住成了大别墅</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>75</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -11817,12 +11816,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -11871,12 +11870,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>红牛资源3</t>
+          <t>TV-天涯资源</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.hongniuzy3.com/api.php/provide/vod</t>
+          <t>https://tyyszy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -11886,13 +11885,11 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>药屋少女的呢喃第三季</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>梦醒时遇见你</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>296</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -11901,24 +11898,24 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>失败:ReadTimeout</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>金鹰资源采集网</t>
+          <t>非凡影视new</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://jyzyapi.com/provide/vod</t>
+          <t>https://api.ffzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -11928,7 +11925,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
+          <t>金缮</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -11948,19 +11945,19 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>非凡影视new</t>
+          <t>红牛资源3</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://api.ffzyapi.com/api.php/provide/vod</t>
+          <t>https://www.hongniuzy3.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -11970,7 +11967,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>我家的弟弟们真是让您费心了</t>
+          <t>药屋少女的呢喃第三季</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -11997,12 +11994,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TV-神马云</t>
+          <t>金鹰资源采集网</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://api.1080zyku.com/inc/apijson.php</t>
+          <t>https://jyzyapi.com/provide/vod</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -12012,11 +12009,13 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>绿头苍蝇</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>707</v>
+          <t>方舟一号第三季</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -12025,24 +12024,24 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>非凡影视</t>
+          <t>豪华资源(代理)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>http://ffzy5.tv/api.php/provide/vod</t>
+          <t>https://pz.v88.qzz.io/?url=https://hhzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -12052,7 +12051,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>我家的弟弟们真是让您费心了</t>
+          <t>方舟一号第三季</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -12072,19 +12071,19 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>索尼-闪电资源</t>
+          <t>🎬量子资源</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://xsd.sdzyapi.com/api.php/provide/vod</t>
+          <t>https://cj.lzcaiji.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -12094,11 +12093,13 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>698</v>
+          <t>霹雳英雄战纪之塗附世界</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -12107,7 +12108,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -12119,12 +12120,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TV-天涯资源</t>
+          <t>🎬豆瓣资源</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://tyyszy.com/api.php/provide/vod</t>
+          <t>https://caiji.dbzy5.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -12134,11 +12135,13 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>改造旧冷库后我住成了大别墅</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>251</v>
+          <t>骑士情缘</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -12147,24 +12150,24 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>失败:ReadTimeout</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>🎬量子资源</t>
+          <t>🎬金鹰点播</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://cj.lzcaiji.com/api.php/provide/vod</t>
+          <t>https://jyzyapi.com/provide/vod/from/jinyingyun/at/json</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -12174,7 +12177,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>霹雳英雄战纪之塗附世界</t>
+          <t>方舟一号第三季</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -12201,12 +12204,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>豪华资源(代理)</t>
+          <t>TV-1080资源</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://pz.v88.qzz.io/?url=https://hhzyapi.com/api.php/provide/vod</t>
+          <t>https://api.1080zyku.com/inc/api_mac10.php</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -12216,13 +12219,11 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>冰雪狙击</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>741</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -12231,24 +12232,24 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>🎬金鹰点播</t>
+          <t>非凡影视</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://jyzyapi.com/provide/vod/from/jinyingyun/at/json</t>
+          <t>http://ffzy5.tv/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -12258,7 +12259,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>方舟一号第三季</t>
+          <t>金缮</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -12278,19 +12279,19 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>🎬豆瓣资源</t>
+          <t>索尼-闪电资源</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>https://caiji.dbzy5.com/api.php/provide/vod</t>
+          <t>https://xsd.sdzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -12300,13 +12301,11 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>骑士情缘</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>可以爱你吗</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>690</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -12315,24 +12314,24 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>未测出</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>🎬快车资源</t>
+          <t>🎬360 资源</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>https://caiji.kuaichezy.org/api.php/provide/vod</t>
+          <t>https://360zyzz.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -12342,11 +12341,11 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
+          <t>Doctor X：白色黑手党时代</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>701</v>
+        <v>610</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -12360,19 +12359,19 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TV-1080资源</t>
+          <t>TV-神马云</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://api.1080zyku.com/inc/api_mac10.php</t>
+          <t>https://api.1080zyku.com/inc/apijson.php</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -12382,11 +12381,11 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>冰雪狙击</t>
+          <t>坠落的大力神</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>563</v>
+        <v>867</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -12395,7 +12394,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>失败:ConnectionError</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -12407,12 +12406,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>🎬360 资源</t>
+          <t>🎬快车资源</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://360zyzz.com/api.php/provide/vod</t>
+          <t>https://caiji.kuaichezy.org/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -12422,11 +12421,11 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Doctor X：白色黑手党时代</t>
+          <t>可以爱你吗</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>613</v>
+        <v>671</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -12440,19 +12439,19 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TV-闪电资源</t>
+          <t>艾旦影视(代理)</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>https://sdzyapi.com/api.php/provide/vod</t>
+          <t>https://pz.v88.qzz.io/?url=https://lovedan.net/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -12462,11 +12461,11 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>可以爱你吗</t>
+          <t>伟大的长征</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>725</v>
+        <v>1411</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -12475,7 +12474,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>失败:ReadTimeout</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -12502,11 +12501,11 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>绿头苍蝇</t>
+          <t>坠落的大力神</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>867</v>
+        <v>2387</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -12527,35 +12526,33 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>艾旦影视(代理)</t>
+          <t>AV-森林资源</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>https://pz.v88.qzz.io/?url=https://lovedan.net/api.php/provide/vod</t>
+          <t>https://slapibf.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>伟大的长征</t>
+          <t>FTHTD-144FALENO学校训练营公共浴池</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>1647</v>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>496</v>
+      </c>
+      <c r="F57" t="n">
+        <v>11334</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>快</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -12567,12 +12564,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>🔞森林资源</t>
+          <t>AV-155资源</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>https://beiyong.slapibf.com/api.php/provide/vod</t>
+          <t>https://155api.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -12582,14 +12579,14 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>FTHTD-144FALENO学校训练营公共浴池</t>
+          <t>内裤走光后宫学园只有我一MOODYZ大崎広浩治沙</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>538</v>
+        <v>52</v>
       </c>
       <c r="F58" t="n">
-        <v>11489</v>
+        <v>10787</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -12605,12 +12602,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>AV-155资源</t>
+          <t>AV-辣椒资源</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>https://155api.com/api.php/provide/vod</t>
+          <t>https://apilj.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -12620,14 +12617,14 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>内裤走光后宫学园只有我一MOODYZ大崎広浩治沙</t>
+          <t>泌尿科的美人女医8人プラネットプラス伊织凉子,管</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>53</v>
+        <v>706</v>
       </c>
       <c r="F59" t="n">
-        <v>11223</v>
+        <v>8946</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -12636,19 +12633,19 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AV-森林资源</t>
+          <t>🔞森林资源</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>https://slapibf.com/api.php/provide/vod</t>
+          <t>https://beiyong.slapibf.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -12662,10 +12659,10 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="F60" t="n">
-        <v>11051</v>
+        <v>8144</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -12681,12 +12678,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>AV-辣椒资源</t>
+          <t>性吧资源</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>https://apilj.com/api.php/provide/vod</t>
+          <t>https://xingba111.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -12696,14 +12693,14 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>泌尿科的美人女医8人プラネットプラス伊织凉子,管</t>
+          <t xml:space="preserve">DASS-303 被派遣按摩師 按摩到敏感部位 </t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>4034</v>
+        <v>575</v>
       </c>
       <c r="F61" t="n">
-        <v>9088</v>
+        <v>7745</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -12712,7 +12709,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
@@ -12738,10 +12735,10 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>456</v>
+        <v>489</v>
       </c>
       <c r="F62" t="n">
-        <v>7835</v>
+        <v>7632</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -12776,10 +12773,10 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>617</v>
+        <v>594</v>
       </c>
       <c r="F63" t="n">
-        <v>7485</v>
+        <v>7439</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -12795,12 +12792,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>性吧资源</t>
+          <t>AV-乐播资源</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>https://xingba111.com/api.php/provide/vod</t>
+          <t>https://lbapi9.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -12810,14 +12807,14 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">DASS-303 被派遣按摩師 按摩到敏感部位 </t>
+          <t>[无码] 苗条人妻床上骚劲爆棚，风骚妩媚狂求内射</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>552</v>
+        <v>915</v>
       </c>
       <c r="F64" t="n">
-        <v>6140</v>
+        <v>4941</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -12833,12 +12830,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AV-乐播资源</t>
+          <t>🔞滴滴资源</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>https://lbapi9.com/api.php/provide/vod</t>
+          <t>https://api.ddapi.cc/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -12848,18 +12845,18 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>[无码] 苗条人妻床上骚劲爆棚，风骚妩媚狂求内射</t>
+          <t>双飞学生妹【蔡萝莉】SM捆绑~白丝足交~强制高潮</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>873</v>
+        <v>324</v>
       </c>
       <c r="F65" t="n">
-        <v>3360</v>
+        <v>885</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>快</t>
+          <t>中</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
@@ -12871,12 +12868,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>🔞滴滴资源</t>
+          <t>🔞豆豆资源</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>https://api.ddapi.cc/api.php/provide/vod</t>
+          <t>https://api.douapi.cc/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -12886,14 +12883,14 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>双飞学生妹【蔡萝莉】SM捆绑~白丝足交~强制高潮</t>
+          <t>美腿玉足控韩国水娃【Hella_cute】顶级吊</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>375</v>
+        <v>343</v>
       </c>
       <c r="F66" t="n">
-        <v>838</v>
+        <v>855</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -12909,12 +12906,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>🔞豆豆资源</t>
+          <t>AV-JKUN资源</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>https://api.douapi.cc/api.php/provide/vod</t>
+          <t>https://jkunzyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -12924,14 +12921,14 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>美腿玉足控韩国水娃【Hella_cute】顶级吊</t>
+          <t>pacopacomama-072023_880-</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>334</v>
+        <v>262</v>
       </c>
       <c r="F67" t="n">
-        <v>805</v>
+        <v>639</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -12947,12 +12944,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>AV-JKUN资源</t>
+          <t>AV-老色逼资源</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>https://jkunzyapi.com/api.php/provide/vod</t>
+          <t>https://apilsbzy1.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -12962,14 +12959,14 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>pacopacomama-072023_880-</t>
+          <t>家庭旅馆偷拍性饥渴嫂子偷情小叔子裤子都没脱就主动</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>58</v>
+        <v>502</v>
       </c>
       <c r="F68" t="n">
-        <v>640</v>
+        <v>442</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -13004,10 +13001,10 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="F69" t="n">
-        <v>463</v>
+        <v>442</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -13023,12 +13020,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>AV-老色逼资源</t>
+          <t>🔞桃花资源</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>https://apilsbzy1.com/api.php/provide/vod</t>
+          <t>https://thzy1.me/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -13038,14 +13035,14 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>家庭旅馆偷拍性饥渴嫂子偷情小叔子裤子都没脱就主动</t>
+          <t>[HornyVerse]_Jane_Doe_Fu</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>231</v>
+        <v>462</v>
       </c>
       <c r="F70" t="n">
-        <v>453</v>
+        <v>375</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -13054,19 +13051,19 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>AV-精品资源</t>
+          <t>AV-奶香香</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>https://www.jingpinx.com/api.php/provide/vod</t>
+          <t>https://Naixxzy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -13076,14 +13073,14 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>純潔的輪舞曲_2</t>
+          <t>[换脸]孙彩瑛 热热的骚逼..</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>397</v>
+        <v>903</v>
       </c>
       <c r="F71" t="n">
-        <v>413</v>
+        <v>335</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -13099,12 +13096,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>AV-奶香香</t>
+          <t>AV-精品资源</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>https://Naixxzy.com/api.php/provide/vod</t>
+          <t>https://www.jingpinx.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -13114,18 +13111,18 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>[换脸]孙彩瑛 热热的骚逼..</t>
+          <t>純潔的輪舞曲_2</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>558</v>
+        <v>480</v>
       </c>
       <c r="F72" t="n">
-        <v>295</v>
+        <v>238</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>慢</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -13137,12 +13134,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>🔞桃花资源</t>
+          <t>🔞-大奶子-</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>https://thzy1.me/api.php/provide/vod</t>
+          <t>https://apidanaizi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -13152,35 +13149,35 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>[HornyVerse]_Jane_Doe_Fu</t>
+          <t>【最新自录-清纯甜美二次元美少女】白裙情趣装罕见</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>611</v>
+        <v>542</v>
       </c>
       <c r="F73" t="n">
-        <v>254</v>
+        <v>222</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>慢</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>🔞-大奶子-</t>
+          <t>AV-奥斯卡资源</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>https://apidanaizi.com/api.php/provide/vod</t>
+          <t>https://aosikazy.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -13190,14 +13187,14 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>【最新自录-清纯甜美二次元美少女】白裙情趣装罕见</t>
+          <t>真实与后妈乱伦9个月</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>563</v>
+        <v>603</v>
       </c>
       <c r="F74" t="n">
-        <v>229</v>
+        <v>173</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -13206,19 +13203,19 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>AV-奥斯卡资源</t>
+          <t>🔞小鸡资源</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>https://aosikazy.com/api.php/provide/vod</t>
+          <t>https://api.xiaojizy.live/provide/vod</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -13228,14 +13225,14 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>真实与后妈乱伦9个月</t>
+          <t>李素英合3</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>624</v>
+        <v>308</v>
       </c>
       <c r="F75" t="n">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -13251,12 +13248,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>🔞小鸡资源</t>
+          <t>🔞黑料资源</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>https://api.xiaojizy.live/provide/vod</t>
+          <t>https://www.heiliaozyapi.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -13266,14 +13263,14 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>李素英合3</t>
+          <t>绿播福利姬女神下海硬控你十分钟一看就高端货超美脸</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>310</v>
+        <v>929</v>
       </c>
       <c r="F76" t="n">
-        <v>169</v>
+        <v>134</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -13308,10 +13305,10 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>1196</v>
+        <v>1284</v>
       </c>
       <c r="F77" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -13327,12 +13324,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>🔞黑料资源</t>
+          <t>AV-souav资源</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>https://www.heiliaozyapi.com/api.php/provide/vod</t>
+          <t>https://api.souavzy.vip/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -13342,35 +13339,37 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>绿播福利姬女神下海硬控你十分钟一看就高端货超美脸</t>
+          <t>白嫩美女月月无套内射初体验</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>981</v>
-      </c>
-      <c r="F78" t="n">
-        <v>118</v>
+        <v>708</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>慢</t>
+          <t>样例过小</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>AV-souav资源</t>
+          <t>黄色资源啊啊</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>https://api.souavzy.vip/api.php/provide/vod</t>
+          <t>https://hsckzy888.com/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -13380,11 +13379,13 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>白嫩美女月月无套内射初体验</t>
-        </is>
-      </c>
-      <c r="E79" t="n">
-        <v>275</v>
+          <t>公共厕所肉便器 我二话 高岭千佳</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -13393,7 +13394,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>样例过小</t>
+          <t>未测出</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -13405,12 +13406,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>黄色资源啊啊</t>
+          <t>🔞黄色仓库</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>https://hsckzy888.com/api.php/provide/vod</t>
+          <t>https://hsckzy.xyz/api.php/provide/vod</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -13447,12 +13448,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>🔞黄色仓库</t>
+          <t>🔞色猫资源</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>https://hsckzy.xyz/api.php/provide/vod</t>
+          <t>https://caiji.semaozy.net/inc/apijson_vod.php/provide/vod</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -13460,11 +13461,7 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>公共厕所肉便器 我二话 高岭千佳</t>
-        </is>
-      </c>
+      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr">
         <is>
           <t>-</t>
@@ -13508,7 +13505,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>456</v>
+        <v>475</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -13521,44 +13518,6 @@
         </is>
       </c>
       <c r="H82" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>🔞色猫资源</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>https://caiji.semaozy.net/inc/apijson_vod.php/provide/vod</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr"/>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>未测出</t>
-        </is>
-      </c>
-      <c r="H83" t="inlineStr">
         <is>
           <t>是</t>
         </is>

</xml_diff>